<commit_message>
Ensure all aquaparks renamed to Akvamir in Excel catalog
</commit_message>
<xml_diff>
--- a/data/БД акции по городам.xlsx
+++ b/data/БД акции по городам.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Аквапарк "Фэнтази"</t>
+          <t>Аквапарк "Аквамир"</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Аквапарк "Фэнтази"</t>
+          <t>Аквапарк "Аквамир"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Аквапарк "Фэнтази"</t>
+          <t>Аквапарк "Аквамир"</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Аквапарк "Фэнтази"</t>
+          <t>Аквапарк "Аквамир"</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">

</xml_diff>